<commit_message>
Projections: season CI back to 95%, weekly stays 80%
Season fantasy floor/ceiling is inherently more predictable (17-game aggregate),
so keep the wider 95% band there; only weekly is narrowed to 80%. Combine-only
change (stacks/base learners untouched).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/projections/def_2026_combined.xlsx
+++ b/projections/def_2026_combined.xlsx
@@ -550,10 +550,10 @@
         <v>120.76</v>
       </c>
       <c r="J2" t="n">
-        <v>72.59999999999999</v>
+        <v>47.1</v>
       </c>
       <c r="K2" t="n">
-        <v>181.79</v>
+        <v>214.1</v>
       </c>
       <c r="L2" t="n">
         <v>42</v>
@@ -610,10 +610,10 @@
         <v>112.98</v>
       </c>
       <c r="J3" t="n">
-        <v>71.47</v>
+        <v>49.5</v>
       </c>
       <c r="K3" t="n">
-        <v>179.6</v>
+        <v>214.86</v>
       </c>
       <c r="L3" t="n">
         <v>44</v>
@@ -670,10 +670,10 @@
         <v>110.81</v>
       </c>
       <c r="J4" t="n">
-        <v>70</v>
+        <v>48.4</v>
       </c>
       <c r="K4" t="n">
-        <v>179.98</v>
+        <v>216.6</v>
       </c>
       <c r="L4" t="n">
         <v>42</v>
@@ -730,10 +730,10 @@
         <v>107.54</v>
       </c>
       <c r="J5" t="n">
-        <v>69</v>
+        <v>48.6</v>
       </c>
       <c r="K5" t="n">
-        <v>176.39</v>
+        <v>212.84</v>
       </c>
       <c r="L5" t="n">
         <v>44</v>
@@ -790,10 +790,10 @@
         <v>106.48</v>
       </c>
       <c r="J6" t="n">
-        <v>67.39</v>
+        <v>46.7</v>
       </c>
       <c r="K6" t="n">
-        <v>173.44</v>
+        <v>208.88</v>
       </c>
       <c r="L6" t="n">
         <v>45</v>
@@ -850,10 +850,10 @@
         <v>104.02</v>
       </c>
       <c r="J7" t="n">
-        <v>66.02</v>
+        <v>45.9</v>
       </c>
       <c r="K7" t="n">
-        <v>169.16</v>
+        <v>203.64</v>
       </c>
       <c r="L7" t="n">
         <v>39</v>
@@ -910,10 +910,10 @@
         <v>103.18</v>
       </c>
       <c r="J8" t="n">
-        <v>67.88</v>
+        <v>49.2</v>
       </c>
       <c r="K8" t="n">
-        <v>174.28</v>
+        <v>211.92</v>
       </c>
       <c r="L8" t="n">
         <v>41</v>
@@ -970,10 +970,10 @@
         <v>103</v>
       </c>
       <c r="J9" t="n">
-        <v>56.12</v>
+        <v>31.3</v>
       </c>
       <c r="K9" t="n">
-        <v>152.14</v>
+        <v>178.16</v>
       </c>
       <c r="L9" t="n">
         <v>39</v>
@@ -1030,10 +1030,10 @@
         <v>100.84</v>
       </c>
       <c r="J10" t="n">
-        <v>53.47</v>
+        <v>28.4</v>
       </c>
       <c r="K10" t="n">
-        <v>172.44</v>
+        <v>210.34</v>
       </c>
       <c r="L10" t="n">
         <v>38</v>
@@ -1090,10 +1090,10 @@
         <v>99.76000000000001</v>
       </c>
       <c r="J11" t="n">
-        <v>65.06999999999999</v>
+        <v>46.7</v>
       </c>
       <c r="K11" t="n">
-        <v>169.21</v>
+        <v>205.98</v>
       </c>
       <c r="L11" t="n">
         <v>44</v>
@@ -1150,10 +1150,10 @@
         <v>99.56</v>
       </c>
       <c r="J12" t="n">
-        <v>54.21</v>
+        <v>30.2</v>
       </c>
       <c r="K12" t="n">
-        <v>147.7</v>
+        <v>173.18</v>
       </c>
       <c r="L12" t="n">
         <v>38</v>
@@ -1210,10 +1210,10 @@
         <v>99.52</v>
       </c>
       <c r="J13" t="n">
-        <v>65.18000000000001</v>
+        <v>47</v>
       </c>
       <c r="K13" t="n">
-        <v>169.84</v>
+        <v>207.06</v>
       </c>
       <c r="L13" t="n">
         <v>39</v>
@@ -1270,10 +1270,10 @@
         <v>98.69</v>
       </c>
       <c r="J14" t="n">
-        <v>52.86</v>
+        <v>28.6</v>
       </c>
       <c r="K14" t="n">
-        <v>146.94</v>
+        <v>172.48</v>
       </c>
       <c r="L14" t="n">
         <v>41</v>
@@ -1330,10 +1330,10 @@
         <v>97.5</v>
       </c>
       <c r="J15" t="n">
-        <v>61.15</v>
+        <v>41.9</v>
       </c>
       <c r="K15" t="n">
-        <v>165.45</v>
+        <v>201.42</v>
       </c>
       <c r="L15" t="n">
         <v>41</v>
@@ -1390,10 +1390,10 @@
         <v>96.83</v>
       </c>
       <c r="J16" t="n">
-        <v>61.44</v>
+        <v>42.7</v>
       </c>
       <c r="K16" t="n">
-        <v>163.19</v>
+        <v>198.32</v>
       </c>
       <c r="L16" t="n">
         <v>40</v>
@@ -1450,10 +1450,10 @@
         <v>96.52</v>
       </c>
       <c r="J17" t="n">
-        <v>52.17</v>
+        <v>28.7</v>
       </c>
       <c r="K17" t="n">
-        <v>143.86</v>
+        <v>168.92</v>
       </c>
       <c r="L17" t="n">
         <v>40</v>
@@ -1510,10 +1510,10 @@
         <v>96.38</v>
       </c>
       <c r="J18" t="n">
-        <v>61.54</v>
+        <v>43.1</v>
       </c>
       <c r="K18" t="n">
-        <v>163.62</v>
+        <v>199.22</v>
       </c>
       <c r="L18" t="n">
         <v>41</v>
@@ -1570,10 +1570,10 @@
         <v>92.67</v>
       </c>
       <c r="J19" t="n">
-        <v>48.82</v>
+        <v>25.6</v>
       </c>
       <c r="K19" t="n">
-        <v>139.48</v>
+        <v>164.26</v>
       </c>
       <c r="L19" t="n">
         <v>39</v>
@@ -1630,10 +1630,10 @@
         <v>92.5</v>
       </c>
       <c r="J20" t="n">
-        <v>48.49</v>
+        <v>25.2</v>
       </c>
       <c r="K20" t="n">
-        <v>139.33</v>
+        <v>164.12</v>
       </c>
       <c r="L20" t="n">
         <v>42</v>
@@ -1690,10 +1690,10 @@
         <v>91.54000000000001</v>
       </c>
       <c r="J21" t="n">
-        <v>47.18</v>
+        <v>23.7</v>
       </c>
       <c r="K21" t="n">
-        <v>138.59</v>
+        <v>163.5</v>
       </c>
       <c r="L21" t="n">
         <v>39</v>
@@ -1750,10 +1750,10 @@
         <v>91.15000000000001</v>
       </c>
       <c r="J22" t="n">
-        <v>48.94</v>
+        <v>26.6</v>
       </c>
       <c r="K22" t="n">
-        <v>125.55</v>
+        <v>143.76</v>
       </c>
       <c r="L22" t="n">
         <v>41</v>
@@ -1810,10 +1810,10 @@
         <v>91</v>
       </c>
       <c r="J23" t="n">
-        <v>57.78</v>
+        <v>40.2</v>
       </c>
       <c r="K23" t="n">
-        <v>160.22</v>
+        <v>196.86</v>
       </c>
       <c r="L23" t="n">
         <v>41</v>
@@ -1870,10 +1870,10 @@
         <v>90.45</v>
       </c>
       <c r="J24" t="n">
-        <v>47.2</v>
+        <v>24.3</v>
       </c>
       <c r="K24" t="n">
-        <v>136.58</v>
+        <v>161</v>
       </c>
       <c r="L24" t="n">
         <v>37</v>
@@ -1930,10 +1930,10 @@
         <v>90.03</v>
       </c>
       <c r="J25" t="n">
-        <v>34.69</v>
+        <v>5.4</v>
       </c>
       <c r="K25" t="n">
-        <v>126.94</v>
+        <v>146.48</v>
       </c>
       <c r="L25" t="n">
         <v>37</v>
@@ -1990,10 +1990,10 @@
         <v>89.73999999999999</v>
       </c>
       <c r="J26" t="n">
-        <v>47.87</v>
+        <v>25.7</v>
       </c>
       <c r="K26" t="n">
-        <v>124.02</v>
+        <v>142.16</v>
       </c>
       <c r="L26" t="n">
         <v>39</v>
@@ -2050,10 +2050,10 @@
         <v>88.77</v>
       </c>
       <c r="J27" t="n">
-        <v>45.57</v>
+        <v>22.7</v>
       </c>
       <c r="K27" t="n">
-        <v>157.13</v>
+        <v>193.32</v>
       </c>
       <c r="L27" t="n">
         <v>38</v>
@@ -2110,10 +2110,10 @@
         <v>87.75</v>
       </c>
       <c r="J28" t="n">
-        <v>46.2</v>
+        <v>24.2</v>
       </c>
       <c r="K28" t="n">
-        <v>121.55</v>
+        <v>139.44</v>
       </c>
       <c r="L28" t="n">
         <v>42</v>
@@ -2170,10 +2170,10 @@
         <v>86.5</v>
       </c>
       <c r="J29" t="n">
-        <v>54.53</v>
+        <v>37.6</v>
       </c>
       <c r="K29" t="n">
-        <v>154.63</v>
+        <v>190.7</v>
       </c>
       <c r="L29" t="n">
         <v>41</v>
@@ -2230,10 +2230,10 @@
         <v>86.28</v>
       </c>
       <c r="J30" t="n">
-        <v>43.14</v>
+        <v>20.3</v>
       </c>
       <c r="K30" t="n">
-        <v>132.27</v>
+        <v>156.62</v>
       </c>
       <c r="L30" t="n">
         <v>39</v>
@@ -2290,10 +2290,10 @@
         <v>84.91</v>
       </c>
       <c r="J31" t="n">
-        <v>43.38</v>
+        <v>21.4</v>
       </c>
       <c r="K31" t="n">
-        <v>152.04</v>
+        <v>187.58</v>
       </c>
       <c r="L31" t="n">
         <v>39</v>
@@ -2350,10 +2350,10 @@
         <v>83.70999999999999</v>
       </c>
       <c r="J32" t="n">
-        <v>42.25</v>
+        <v>20.3</v>
       </c>
       <c r="K32" t="n">
-        <v>117.25</v>
+        <v>135</v>
       </c>
       <c r="L32" t="n">
         <v>38</v>
@@ -2410,10 +2410,10 @@
         <v>83.02</v>
       </c>
       <c r="J33" t="n">
-        <v>41.16</v>
+        <v>19</v>
       </c>
       <c r="K33" t="n">
-        <v>116.82</v>
+        <v>134.72</v>
       </c>
       <c r="L33" t="n">
         <v>36</v>

</xml_diff>